<commit_message>
Treat 0 in API volume indices as missing (construction 2010 showed -100%)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019gDGnwpLiCWtJjrgA1nuow
</commit_message>
<xml_diff>
--- a/data/history/long/history_long.xlsx
+++ b/data/history/long/history_long.xlsx
@@ -6027,9 +6027,6 @@
       <c r="A66" t="s">
         <v>65</v>
       </c>
-      <c r="G66">
-        <v>-100</v>
-      </c>
       <c r="H66">
         <v>20.96666666666667</v>
       </c>
@@ -7287,12 +7284,6 @@
       <c r="A93" t="s">
         <v>92</v>
       </c>
-      <c r="J93">
-        <v>-100</v>
-      </c>
-      <c r="K93">
-        <v>-100</v>
-      </c>
       <c r="L93">
         <v>-27.40833333333333</v>
       </c>
@@ -7331,12 +7322,6 @@
       <c r="A94" t="s">
         <v>93</v>
       </c>
-      <c r="J94">
-        <v>-100</v>
-      </c>
-      <c r="K94">
-        <v>-100</v>
-      </c>
       <c r="L94">
         <v>-3.066666666666666</v>
       </c>
@@ -7374,12 +7359,6 @@
     <row r="95" spans="1:22">
       <c r="A95" t="s">
         <v>94</v>
-      </c>
-      <c r="J95">
-        <v>-100</v>
-      </c>
-      <c r="K95">
-        <v>-100</v>
       </c>
       <c r="L95">
         <v>-6.683333333333334</v>
@@ -13218,13 +13197,13 @@
         <v>450</v>
       </c>
       <c r="F65">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="G65">
         <v>2025</v>
       </c>
       <c r="H65">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -13920,13 +13899,13 @@
         <v>469</v>
       </c>
       <c r="F92">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="G92">
         <v>2025</v>
       </c>
       <c r="H92">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -13946,13 +13925,13 @@
         <v>470</v>
       </c>
       <c r="F93">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="G93">
         <v>2025</v>
       </c>
       <c r="H93">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -13972,13 +13951,13 @@
         <v>471</v>
       </c>
       <c r="F94">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="G94">
         <v>2025</v>
       </c>
       <c r="H94">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -29354,18 +29333,6 @@
       <c r="A37" t="s">
         <v>65</v>
       </c>
-      <c r="V37">
-        <v>-100</v>
-      </c>
-      <c r="W37">
-        <v>-100</v>
-      </c>
-      <c r="X37">
-        <v>-100</v>
-      </c>
-      <c r="Y37">
-        <v>-100</v>
-      </c>
       <c r="Z37">
         <v>18.53333333333333</v>
       </c>
@@ -34181,30 +34148,6 @@
       <c r="A64" t="s">
         <v>92</v>
       </c>
-      <c r="AH64">
-        <v>-100</v>
-      </c>
-      <c r="AI64">
-        <v>-100</v>
-      </c>
-      <c r="AJ64">
-        <v>-100</v>
-      </c>
-      <c r="AK64">
-        <v>-100</v>
-      </c>
-      <c r="AL64">
-        <v>-100</v>
-      </c>
-      <c r="AM64">
-        <v>-100</v>
-      </c>
-      <c r="AN64">
-        <v>-100</v>
-      </c>
-      <c r="AO64">
-        <v>-100</v>
-      </c>
       <c r="AP64">
         <v>-55.7</v>
       </c>
@@ -34348,30 +34291,6 @@
       <c r="A65" t="s">
         <v>93</v>
       </c>
-      <c r="AH65">
-        <v>-100</v>
-      </c>
-      <c r="AI65">
-        <v>-100</v>
-      </c>
-      <c r="AJ65">
-        <v>-100</v>
-      </c>
-      <c r="AK65">
-        <v>-100</v>
-      </c>
-      <c r="AL65">
-        <v>-100</v>
-      </c>
-      <c r="AM65">
-        <v>-100</v>
-      </c>
-      <c r="AN65">
-        <v>-100</v>
-      </c>
-      <c r="AO65">
-        <v>-100</v>
-      </c>
       <c r="AP65">
         <v>-2.800000000000002</v>
       </c>
@@ -34514,30 +34433,6 @@
     <row r="66" spans="1:88">
       <c r="A66" t="s">
         <v>94</v>
-      </c>
-      <c r="AH66">
-        <v>-100</v>
-      </c>
-      <c r="AI66">
-        <v>-100</v>
-      </c>
-      <c r="AJ66">
-        <v>-100</v>
-      </c>
-      <c r="AK66">
-        <v>-100</v>
-      </c>
-      <c r="AL66">
-        <v>-100</v>
-      </c>
-      <c r="AM66">
-        <v>-100</v>
-      </c>
-      <c r="AN66">
-        <v>-100</v>
-      </c>
-      <c r="AO66">
-        <v>-100</v>
       </c>
       <c r="AP66">
         <v>-14.7</v>
@@ -48672,13 +48567,13 @@
         <v>648</v>
       </c>
       <c r="F66" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="G66" t="s">
         <v>595</v>
       </c>
       <c r="H66">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I66" t="s">
         <v>691</v>
@@ -49455,13 +49350,13 @@
         <v>667</v>
       </c>
       <c r="F93" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G93" t="s">
         <v>595</v>
       </c>
       <c r="H93">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I93" t="s">
         <v>691</v>
@@ -49484,13 +49379,13 @@
         <v>668</v>
       </c>
       <c r="F94" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G94" t="s">
         <v>595</v>
       </c>
       <c r="H94">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I94" t="s">
         <v>691</v>
@@ -49513,13 +49408,13 @@
         <v>669</v>
       </c>
       <c r="F95" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G95" t="s">
         <v>595</v>
       </c>
       <c r="H95">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I95" t="s">
         <v>691</v>

</xml_diff>

<commit_message>
Treat 0 in API volume indices as missing (construction 2010 showed -100%) (#21)
Claude-Session: https://claude.ai/code/session_019gDGnwpLiCWtJjrgA1nuow

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/history/long/history_long.xlsx
+++ b/data/history/long/history_long.xlsx
@@ -6027,9 +6027,6 @@
       <c r="A66" t="s">
         <v>65</v>
       </c>
-      <c r="G66">
-        <v>-100</v>
-      </c>
       <c r="H66">
         <v>20.96666666666667</v>
       </c>
@@ -7287,12 +7284,6 @@
       <c r="A93" t="s">
         <v>92</v>
       </c>
-      <c r="J93">
-        <v>-100</v>
-      </c>
-      <c r="K93">
-        <v>-100</v>
-      </c>
       <c r="L93">
         <v>-27.40833333333333</v>
       </c>
@@ -7331,12 +7322,6 @@
       <c r="A94" t="s">
         <v>93</v>
       </c>
-      <c r="J94">
-        <v>-100</v>
-      </c>
-      <c r="K94">
-        <v>-100</v>
-      </c>
       <c r="L94">
         <v>-3.066666666666666</v>
       </c>
@@ -7374,12 +7359,6 @@
     <row r="95" spans="1:22">
       <c r="A95" t="s">
         <v>94</v>
-      </c>
-      <c r="J95">
-        <v>-100</v>
-      </c>
-      <c r="K95">
-        <v>-100</v>
       </c>
       <c r="L95">
         <v>-6.683333333333334</v>
@@ -13218,13 +13197,13 @@
         <v>450</v>
       </c>
       <c r="F65">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="G65">
         <v>2025</v>
       </c>
       <c r="H65">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -13920,13 +13899,13 @@
         <v>469</v>
       </c>
       <c r="F92">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="G92">
         <v>2025</v>
       </c>
       <c r="H92">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -13946,13 +13925,13 @@
         <v>470</v>
       </c>
       <c r="F93">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="G93">
         <v>2025</v>
       </c>
       <c r="H93">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -13972,13 +13951,13 @@
         <v>471</v>
       </c>
       <c r="F94">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="G94">
         <v>2025</v>
       </c>
       <c r="H94">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -29354,18 +29333,6 @@
       <c r="A37" t="s">
         <v>65</v>
       </c>
-      <c r="V37">
-        <v>-100</v>
-      </c>
-      <c r="W37">
-        <v>-100</v>
-      </c>
-      <c r="X37">
-        <v>-100</v>
-      </c>
-      <c r="Y37">
-        <v>-100</v>
-      </c>
       <c r="Z37">
         <v>18.53333333333333</v>
       </c>
@@ -34181,30 +34148,6 @@
       <c r="A64" t="s">
         <v>92</v>
       </c>
-      <c r="AH64">
-        <v>-100</v>
-      </c>
-      <c r="AI64">
-        <v>-100</v>
-      </c>
-      <c r="AJ64">
-        <v>-100</v>
-      </c>
-      <c r="AK64">
-        <v>-100</v>
-      </c>
-      <c r="AL64">
-        <v>-100</v>
-      </c>
-      <c r="AM64">
-        <v>-100</v>
-      </c>
-      <c r="AN64">
-        <v>-100</v>
-      </c>
-      <c r="AO64">
-        <v>-100</v>
-      </c>
       <c r="AP64">
         <v>-55.7</v>
       </c>
@@ -34348,30 +34291,6 @@
       <c r="A65" t="s">
         <v>93</v>
       </c>
-      <c r="AH65">
-        <v>-100</v>
-      </c>
-      <c r="AI65">
-        <v>-100</v>
-      </c>
-      <c r="AJ65">
-        <v>-100</v>
-      </c>
-      <c r="AK65">
-        <v>-100</v>
-      </c>
-      <c r="AL65">
-        <v>-100</v>
-      </c>
-      <c r="AM65">
-        <v>-100</v>
-      </c>
-      <c r="AN65">
-        <v>-100</v>
-      </c>
-      <c r="AO65">
-        <v>-100</v>
-      </c>
       <c r="AP65">
         <v>-2.800000000000002</v>
       </c>
@@ -34514,30 +34433,6 @@
     <row r="66" spans="1:88">
       <c r="A66" t="s">
         <v>94</v>
-      </c>
-      <c r="AH66">
-        <v>-100</v>
-      </c>
-      <c r="AI66">
-        <v>-100</v>
-      </c>
-      <c r="AJ66">
-        <v>-100</v>
-      </c>
-      <c r="AK66">
-        <v>-100</v>
-      </c>
-      <c r="AL66">
-        <v>-100</v>
-      </c>
-      <c r="AM66">
-        <v>-100</v>
-      </c>
-      <c r="AN66">
-        <v>-100</v>
-      </c>
-      <c r="AO66">
-        <v>-100</v>
       </c>
       <c r="AP66">
         <v>-14.7</v>
@@ -48672,13 +48567,13 @@
         <v>648</v>
       </c>
       <c r="F66" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="G66" t="s">
         <v>595</v>
       </c>
       <c r="H66">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I66" t="s">
         <v>691</v>
@@ -49455,13 +49350,13 @@
         <v>667</v>
       </c>
       <c r="F93" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G93" t="s">
         <v>595</v>
       </c>
       <c r="H93">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I93" t="s">
         <v>691</v>
@@ -49484,13 +49379,13 @@
         <v>668</v>
       </c>
       <c r="F94" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G94" t="s">
         <v>595</v>
       </c>
       <c r="H94">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I94" t="s">
         <v>691</v>
@@ -49513,13 +49408,13 @@
         <v>669</v>
       </c>
       <c r="F95" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G95" t="s">
         <v>595</v>
       </c>
       <c r="H95">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="I95" t="s">
         <v>691</v>

</xml_diff>

<commit_message>
Drop MacroStat CPI years copied from the previous year
MacroStat's CPI sheet repeats 2011 as 2012; such years are now dropped so
component y/y for 2012-2013 is missing instead of zero.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019gDGnwpLiCWtJjrgA1nuow
</commit_message>
<xml_diff>
--- a/data/history/long/history_long.xlsx
+++ b/data/history/long/history_long.xlsx
@@ -8187,12 +8187,6 @@
       <c r="H111">
         <v>22.9268</v>
       </c>
-      <c r="I111">
-        <v>22.9268</v>
-      </c>
-      <c r="J111">
-        <v>0</v>
-      </c>
       <c r="K111">
         <v>11.3</v>
       </c>
@@ -8228,12 +8222,6 @@
       <c r="H112">
         <v>0</v>
       </c>
-      <c r="I112">
-        <v>0</v>
-      </c>
-      <c r="J112">
-        <v>0</v>
-      </c>
       <c r="K112">
         <v>62.80000000000001</v>
       </c>
@@ -8269,12 +8257,6 @@
       <c r="H113">
         <v>15.09967044335447</v>
       </c>
-      <c r="I113">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="J113">
-        <v>-0.223565590534065</v>
-      </c>
       <c r="K113">
         <v>46.87817633473585</v>
       </c>
@@ -8310,12 +8292,6 @@
       <c r="H114">
         <v>3.555927309945545</v>
       </c>
-      <c r="I114">
-        <v>3.555927309945545</v>
-      </c>
-      <c r="J114">
-        <v>0.9033061050990625</v>
-      </c>
       <c r="K114">
         <v>27.21676429317348</v>
       </c>
@@ -8353,12 +8329,6 @@
       </c>
       <c r="H115">
         <v>30.87659038941771</v>
-      </c>
-      <c r="I115">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="J115">
-        <v>-3.64978448421158</v>
       </c>
       <c r="K115">
         <v>60.66156020913212</v>
@@ -14373,7 +14343,7 @@
         <v>2022</v>
       </c>
       <c r="H110">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -14399,7 +14369,7 @@
         <v>2022</v>
       </c>
       <c r="H111">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -14425,7 +14395,7 @@
         <v>2022</v>
       </c>
       <c r="H112">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -14451,7 +14421,7 @@
         <v>2025</v>
       </c>
       <c r="H113">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -14477,7 +14447,7 @@
         <v>2022</v>
       </c>
       <c r="H114">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -37616,27 +37586,6 @@
       <c r="AC82">
         <v>22.9268</v>
       </c>
-      <c r="AD82">
-        <v>22.9268</v>
-      </c>
-      <c r="AE82">
-        <v>22.9268</v>
-      </c>
-      <c r="AF82">
-        <v>22.9268</v>
-      </c>
-      <c r="AG82">
-        <v>22.9268</v>
-      </c>
-      <c r="AH82">
-        <v>15.10000000000001</v>
-      </c>
-      <c r="AI82">
-        <v>0</v>
-      </c>
-      <c r="AJ82">
-        <v>0</v>
-      </c>
       <c r="AK82">
         <v>0</v>
       </c>
@@ -37786,27 +37735,6 @@
       <c r="AC83">
         <v>0</v>
       </c>
-      <c r="AD83">
-        <v>0</v>
-      </c>
-      <c r="AE83">
-        <v>0</v>
-      </c>
-      <c r="AF83">
-        <v>0</v>
-      </c>
-      <c r="AG83">
-        <v>0</v>
-      </c>
-      <c r="AH83">
-        <v>0</v>
-      </c>
-      <c r="AI83">
-        <v>0</v>
-      </c>
-      <c r="AJ83">
-        <v>0</v>
-      </c>
       <c r="AK83">
         <v>0</v>
       </c>
@@ -37956,27 +37884,6 @@
       <c r="AC84">
         <v>15.09967044335447</v>
       </c>
-      <c r="AD84">
-        <v>15.09967044335451</v>
-      </c>
-      <c r="AE84">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="AF84">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="AG84">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="AH84">
-        <v>0.2789504710609521</v>
-      </c>
-      <c r="AI84">
-        <v>1.187615256060326</v>
-      </c>
-      <c r="AJ84">
-        <v>1.187615256060326</v>
-      </c>
       <c r="AK84">
         <v>-0.223565590534065</v>
       </c>
@@ -38126,27 +38033,6 @@
       <c r="AC85">
         <v>3.555927309945545</v>
       </c>
-      <c r="AD85">
-        <v>3.555927309945488</v>
-      </c>
-      <c r="AE85">
-        <v>3.555927309945488</v>
-      </c>
-      <c r="AF85">
-        <v>3.555927309945488</v>
-      </c>
-      <c r="AG85">
-        <v>3.555927309945545</v>
-      </c>
-      <c r="AH85">
-        <v>3.143148635187671</v>
-      </c>
-      <c r="AI85">
-        <v>2.221318015973026</v>
-      </c>
-      <c r="AJ85">
-        <v>1.611245316801345</v>
-      </c>
       <c r="AK85">
         <v>0.9033061050990625</v>
       </c>
@@ -38307,27 +38193,6 @@
       </c>
       <c r="AC86">
         <v>30.87659038941771</v>
-      </c>
-      <c r="AD86">
-        <v>30.87659038941769</v>
-      </c>
-      <c r="AE86">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="AF86">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="AG86">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="AH86">
-        <v>8.375096230444328</v>
-      </c>
-      <c r="AI86">
-        <v>-1.596550984285486</v>
-      </c>
-      <c r="AJ86">
-        <v>-1.596354766042197</v>
       </c>
       <c r="AK86">
         <v>-3.64978448421158</v>
@@ -49878,7 +49743,7 @@
         <v>596</v>
       </c>
       <c r="H111">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I111" t="s">
         <v>691</v>
@@ -49907,7 +49772,7 @@
         <v>596</v>
       </c>
       <c r="H112">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I112" t="s">
         <v>691</v>
@@ -49936,7 +49801,7 @@
         <v>596</v>
       </c>
       <c r="H113">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I113" t="s">
         <v>691</v>
@@ -49965,7 +49830,7 @@
         <v>596</v>
       </c>
       <c r="H114">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="I114" t="s">
         <v>691</v>
@@ -49994,7 +49859,7 @@
         <v>596</v>
       </c>
       <c r="H115">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="I115" t="s">
         <v>691</v>

</xml_diff>

<commit_message>
Drop MacroStat CPI years copied from the previous year (#23)
MacroStat's CPI sheet repeats 2011 as 2012; such years are now dropped so
component y/y for 2012-2013 is missing instead of zero.


Claude-Session: https://claude.ai/code/session_019gDGnwpLiCWtJjrgA1nuow

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/history/long/history_long.xlsx
+++ b/data/history/long/history_long.xlsx
@@ -8187,12 +8187,6 @@
       <c r="H111">
         <v>22.9268</v>
       </c>
-      <c r="I111">
-        <v>22.9268</v>
-      </c>
-      <c r="J111">
-        <v>0</v>
-      </c>
       <c r="K111">
         <v>11.3</v>
       </c>
@@ -8228,12 +8222,6 @@
       <c r="H112">
         <v>0</v>
       </c>
-      <c r="I112">
-        <v>0</v>
-      </c>
-      <c r="J112">
-        <v>0</v>
-      </c>
       <c r="K112">
         <v>62.80000000000001</v>
       </c>
@@ -8269,12 +8257,6 @@
       <c r="H113">
         <v>15.09967044335447</v>
       </c>
-      <c r="I113">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="J113">
-        <v>-0.223565590534065</v>
-      </c>
       <c r="K113">
         <v>46.87817633473585</v>
       </c>
@@ -8310,12 +8292,6 @@
       <c r="H114">
         <v>3.555927309945545</v>
       </c>
-      <c r="I114">
-        <v>3.555927309945545</v>
-      </c>
-      <c r="J114">
-        <v>0.9033061050990625</v>
-      </c>
       <c r="K114">
         <v>27.21676429317348</v>
       </c>
@@ -8353,12 +8329,6 @@
       </c>
       <c r="H115">
         <v>30.87659038941771</v>
-      </c>
-      <c r="I115">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="J115">
-        <v>-3.64978448421158</v>
       </c>
       <c r="K115">
         <v>60.66156020913212</v>
@@ -14373,7 +14343,7 @@
         <v>2022</v>
       </c>
       <c r="H110">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -14399,7 +14369,7 @@
         <v>2022</v>
       </c>
       <c r="H111">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -14425,7 +14395,7 @@
         <v>2022</v>
       </c>
       <c r="H112">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -14451,7 +14421,7 @@
         <v>2025</v>
       </c>
       <c r="H113">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -14477,7 +14447,7 @@
         <v>2022</v>
       </c>
       <c r="H114">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -37616,27 +37586,6 @@
       <c r="AC82">
         <v>22.9268</v>
       </c>
-      <c r="AD82">
-        <v>22.9268</v>
-      </c>
-      <c r="AE82">
-        <v>22.9268</v>
-      </c>
-      <c r="AF82">
-        <v>22.9268</v>
-      </c>
-      <c r="AG82">
-        <v>22.9268</v>
-      </c>
-      <c r="AH82">
-        <v>15.10000000000001</v>
-      </c>
-      <c r="AI82">
-        <v>0</v>
-      </c>
-      <c r="AJ82">
-        <v>0</v>
-      </c>
       <c r="AK82">
         <v>0</v>
       </c>
@@ -37786,27 +37735,6 @@
       <c r="AC83">
         <v>0</v>
       </c>
-      <c r="AD83">
-        <v>0</v>
-      </c>
-      <c r="AE83">
-        <v>0</v>
-      </c>
-      <c r="AF83">
-        <v>0</v>
-      </c>
-      <c r="AG83">
-        <v>0</v>
-      </c>
-      <c r="AH83">
-        <v>0</v>
-      </c>
-      <c r="AI83">
-        <v>0</v>
-      </c>
-      <c r="AJ83">
-        <v>0</v>
-      </c>
       <c r="AK83">
         <v>0</v>
       </c>
@@ -37956,27 +37884,6 @@
       <c r="AC84">
         <v>15.09967044335447</v>
       </c>
-      <c r="AD84">
-        <v>15.09967044335451</v>
-      </c>
-      <c r="AE84">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="AF84">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="AG84">
-        <v>15.09967044335447</v>
-      </c>
-      <c r="AH84">
-        <v>0.2789504710609521</v>
-      </c>
-      <c r="AI84">
-        <v>1.187615256060326</v>
-      </c>
-      <c r="AJ84">
-        <v>1.187615256060326</v>
-      </c>
       <c r="AK84">
         <v>-0.223565590534065</v>
       </c>
@@ -38126,27 +38033,6 @@
       <c r="AC85">
         <v>3.555927309945545</v>
       </c>
-      <c r="AD85">
-        <v>3.555927309945488</v>
-      </c>
-      <c r="AE85">
-        <v>3.555927309945488</v>
-      </c>
-      <c r="AF85">
-        <v>3.555927309945488</v>
-      </c>
-      <c r="AG85">
-        <v>3.555927309945545</v>
-      </c>
-      <c r="AH85">
-        <v>3.143148635187671</v>
-      </c>
-      <c r="AI85">
-        <v>2.221318015973026</v>
-      </c>
-      <c r="AJ85">
-        <v>1.611245316801345</v>
-      </c>
       <c r="AK85">
         <v>0.9033061050990625</v>
       </c>
@@ -38307,27 +38193,6 @@
       </c>
       <c r="AC86">
         <v>30.87659038941771</v>
-      </c>
-      <c r="AD86">
-        <v>30.87659038941769</v>
-      </c>
-      <c r="AE86">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="AF86">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="AG86">
-        <v>30.87659038941771</v>
-      </c>
-      <c r="AH86">
-        <v>8.375096230444328</v>
-      </c>
-      <c r="AI86">
-        <v>-1.596550984285486</v>
-      </c>
-      <c r="AJ86">
-        <v>-1.596354766042197</v>
       </c>
       <c r="AK86">
         <v>-3.64978448421158</v>
@@ -49878,7 +49743,7 @@
         <v>596</v>
       </c>
       <c r="H111">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I111" t="s">
         <v>691</v>
@@ -49907,7 +49772,7 @@
         <v>596</v>
       </c>
       <c r="H112">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I112" t="s">
         <v>691</v>
@@ -49936,7 +49801,7 @@
         <v>596</v>
       </c>
       <c r="H113">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I113" t="s">
         <v>691</v>
@@ -49965,7 +49830,7 @@
         <v>596</v>
       </c>
       <c r="H114">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="I114" t="s">
         <v>691</v>
@@ -49994,7 +49859,7 @@
         <v>596</v>
       </c>
       <c r="H115">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="I115" t="s">
         <v>691</v>

</xml_diff>